<commit_message>
added && implemented util "writeYearsToColumns"
</commit_message>
<xml_diff>
--- a/skuMetrics.xlsx
+++ b/skuMetrics.xlsx
@@ -465,15 +465,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A159"/>
+  <dimension ref="A1:C159"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
+    <col min="2" max="3" width="20" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
+      </c>
+      <c r="B1" s="1">
+        <v>2025</v>
+      </c>
+      <c r="C1" s="1">
+        <v>2026</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
updated writeSkuDataToCells: added third arg skuDataIndent, added year to each sku
</commit_message>
<xml_diff>
--- a/skuMetrics.xlsx
+++ b/skuMetrics.xlsx
@@ -469,33 +469,38 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="3" width="20" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1">
+      <c r="B1">
         <v>2025</v>
       </c>
-      <c r="C1" s="1">
+      <c r="C1">
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
+      </c>
+      <c r="B2">
+        <v>22</v>
+      </c>
+      <c r="C2">
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="1">
-        <v>0</v>
-      </c>
-      <c r="C3" s="1">
+      <c r="B3">
+        <v>-1072.65</v>
+      </c>
+      <c r="C3">
         <v>0</v>
       </c>
     </row>
@@ -503,10 +508,10 @@
       <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="1">
-        <v>0</v>
-      </c>
-      <c r="C4" s="1">
+      <c r="B4">
+        <v>0</v>
+      </c>
+      <c r="C4">
         <v>0</v>
       </c>
     </row>
@@ -514,10 +519,10 @@
       <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="1">
-        <v>0</v>
-      </c>
-      <c r="C5" s="1">
+      <c r="B5">
+        <v>5981.06</v>
+      </c>
+      <c r="C5">
         <v>0</v>
       </c>
     </row>
@@ -525,10 +530,10 @@
       <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="1">
-        <v>0</v>
-      </c>
-      <c r="C6" s="1">
+      <c r="B6">
+        <v>0</v>
+      </c>
+      <c r="C6">
         <v>0</v>
       </c>
     </row>
@@ -536,10 +541,10 @@
       <c r="A7" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="1">
-        <v>0</v>
-      </c>
-      <c r="C7" s="1">
+      <c r="B7">
+        <v>6656.96</v>
+      </c>
+      <c r="C7">
         <v>0</v>
       </c>
     </row>
@@ -547,10 +552,10 @@
       <c r="A8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="1">
-        <v>0</v>
-      </c>
-      <c r="C8" s="1">
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8">
         <v>0</v>
       </c>
     </row>
@@ -558,10 +563,10 @@
       <c r="A9" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="1">
-        <v>0</v>
-      </c>
-      <c r="C9" s="1">
+      <c r="B9">
+        <v>165.48</v>
+      </c>
+      <c r="C9">
         <v>0</v>
       </c>
     </row>
@@ -569,10 +574,10 @@
       <c r="A10" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="1">
-        <v>0</v>
-      </c>
-      <c r="C10" s="1">
+      <c r="B10">
+        <v>1622.5</v>
+      </c>
+      <c r="C10">
         <v>0</v>
       </c>
     </row>
@@ -580,10 +585,10 @@
       <c r="A11" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="1">
-        <v>0</v>
-      </c>
-      <c r="C11" s="1">
+      <c r="B11">
+        <v>0</v>
+      </c>
+      <c r="C11">
         <v>0</v>
       </c>
     </row>
@@ -591,10 +596,10 @@
       <c r="A12" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="1">
-        <v>0</v>
-      </c>
-      <c r="C12" s="1">
+      <c r="B12">
+        <v>238.91</v>
+      </c>
+      <c r="C12">
         <v>0</v>
       </c>
     </row>
@@ -602,10 +607,10 @@
       <c r="A13" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="1">
-        <v>0</v>
-      </c>
-      <c r="C13" s="1">
+      <c r="B13">
+        <v>0</v>
+      </c>
+      <c r="C13">
         <v>0</v>
       </c>
     </row>
@@ -613,10 +618,10 @@
       <c r="A14" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="1">
-        <v>0</v>
-      </c>
-      <c r="C14" s="1">
+      <c r="B14">
+        <v>3222.82</v>
+      </c>
+      <c r="C14">
         <v>0</v>
       </c>
     </row>
@@ -624,694 +629,1496 @@
       <c r="A15" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="1">
-        <v>0</v>
-      </c>
-      <c r="C15" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B16" s="1">
-        <v>0</v>
-      </c>
-      <c r="C16" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B15">
+        <v>48.41</v>
+      </c>
+      <c r="C15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B17">
+        <v>2025</v>
+      </c>
+      <c r="C17">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B19">
+        <v>3.4</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B20">
+        <v>0</v>
+      </c>
+      <c r="C20">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B21">
+        <v>375.9</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B22">
+        <v>0</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B23">
+        <v>340</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B24">
+        <v>0</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B25">
+        <v>0.4</v>
+      </c>
+      <c r="C25">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B26">
+        <v>83.2</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B27">
+        <v>0</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B28">
+        <v>18.03</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B29">
+        <v>0</v>
+      </c>
+      <c r="C29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B30">
+        <v>158.87</v>
+      </c>
+      <c r="C30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B31">
+        <v>46.73</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B33">
+        <v>2025</v>
+      </c>
+      <c r="C33">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B34">
+        <v>0</v>
+      </c>
+      <c r="C34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B35">
+        <v>0</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B36">
+        <v>0</v>
+      </c>
+      <c r="C36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B37">
+        <v>0</v>
+      </c>
+      <c r="C37">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B38">
+        <v>0</v>
+      </c>
+      <c r="C38">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B39">
+        <v>0</v>
+      </c>
+      <c r="C39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B40">
+        <v>0</v>
+      </c>
+      <c r="C40">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B41">
+        <v>0</v>
+      </c>
+      <c r="C41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B42">
+        <v>0</v>
+      </c>
+      <c r="C42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B43">
+        <v>0</v>
+      </c>
+      <c r="C43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B44">
+        <v>0</v>
+      </c>
+      <c r="C44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B45">
+        <v>0</v>
+      </c>
+      <c r="C45">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B46">
+        <v>0</v>
+      </c>
+      <c r="C46">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B47">
+        <v>0</v>
+      </c>
+      <c r="C47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B49">
+        <v>2025</v>
+      </c>
+      <c r="C49">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B50">
+        <v>0</v>
+      </c>
+      <c r="C50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B51">
+        <v>0</v>
+      </c>
+      <c r="C51">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B52">
+        <v>0</v>
+      </c>
+      <c r="C52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B53">
+        <v>0</v>
+      </c>
+      <c r="C53">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B54">
+        <v>0</v>
+      </c>
+      <c r="C54">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B55">
+        <v>0</v>
+      </c>
+      <c r="C55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B56">
+        <v>0</v>
+      </c>
+      <c r="C56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B57">
+        <v>0</v>
+      </c>
+      <c r="C57">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B58">
+        <v>0</v>
+      </c>
+      <c r="C58">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B59">
+        <v>0</v>
+      </c>
+      <c r="C59">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B60">
+        <v>0</v>
+      </c>
+      <c r="C60">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B61">
+        <v>0</v>
+      </c>
+      <c r="C61">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B62">
+        <v>0</v>
+      </c>
+      <c r="C62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B63">
+        <v>0</v>
+      </c>
+      <c r="C63">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B65">
+        <v>2025</v>
+      </c>
+      <c r="C65">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B66">
+        <v>1</v>
+      </c>
+      <c r="C66">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B67">
+        <v>1.83</v>
+      </c>
+      <c r="C67">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B68">
+        <v>0</v>
+      </c>
+      <c r="C68">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B69">
+        <v>231.35</v>
+      </c>
+      <c r="C69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B70">
+        <v>0</v>
+      </c>
+      <c r="C70">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B71">
+        <v>183</v>
+      </c>
+      <c r="C71">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B72">
+        <v>0</v>
+      </c>
+      <c r="C72">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B73">
+        <v>0</v>
+      </c>
+      <c r="C73">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B74">
+        <v>42.9</v>
+      </c>
+      <c r="C74">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B75">
+        <v>0</v>
+      </c>
+      <c r="C75">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B76">
+        <v>13.24</v>
+      </c>
+      <c r="C76">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B77">
+        <v>0</v>
+      </c>
+      <c r="C77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B78">
+        <v>117.38</v>
+      </c>
+      <c r="C78">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B79">
+        <v>64.14</v>
+      </c>
+      <c r="C79">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B81">
+        <v>2025</v>
+      </c>
+      <c r="C81">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B82">
+        <v>1</v>
+      </c>
+      <c r="C82">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B83">
+        <v>1.83</v>
+      </c>
+      <c r="C83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B84">
+        <v>0</v>
+      </c>
+      <c r="C84">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B85">
+        <v>231.35</v>
+      </c>
+      <c r="C85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B86">
+        <v>0</v>
+      </c>
+      <c r="C86">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B87">
+        <v>183</v>
+      </c>
+      <c r="C87">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B88">
+        <v>0</v>
+      </c>
+      <c r="C88">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B89">
+        <v>0</v>
+      </c>
+      <c r="C89">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B90">
+        <v>42.9</v>
+      </c>
+      <c r="C90">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B91">
+        <v>0</v>
+      </c>
+      <c r="C91">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B92">
+        <v>13.24</v>
+      </c>
+      <c r="C92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B93">
+        <v>0</v>
+      </c>
+      <c r="C93">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B94">
+        <v>117.38</v>
+      </c>
+      <c r="C94">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B95">
+        <v>64.14</v>
+      </c>
+      <c r="C95">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B97">
+        <v>2025</v>
+      </c>
+      <c r="C97">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B98">
+        <v>14</v>
+      </c>
+      <c r="C98">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B99">
+        <v>-606.4</v>
+      </c>
+      <c r="C99">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B100">
+        <v>0</v>
+      </c>
+      <c r="C100">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B101">
+        <v>3215.06</v>
+      </c>
+      <c r="C101">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B102">
+        <v>0</v>
+      </c>
+      <c r="C102">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B103">
+        <v>4048</v>
+      </c>
+      <c r="C103">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B104">
+        <v>3</v>
+      </c>
+      <c r="C104">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B105">
+        <v>176.96</v>
+      </c>
+      <c r="C105">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B106">
+        <v>1151.3</v>
+      </c>
+      <c r="C106">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B107">
+        <v>0</v>
+      </c>
+      <c r="C107">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B108">
+        <v>110.28</v>
+      </c>
+      <c r="C108">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B109">
+        <v>0</v>
+      </c>
+      <c r="C109">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B110">
+        <v>1598.92</v>
+      </c>
+      <c r="C110">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B111">
+        <v>39.5</v>
+      </c>
+      <c r="C111">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B113">
+        <v>2025</v>
+      </c>
+      <c r="C113">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B114">
+        <v>0</v>
+      </c>
+      <c r="C114">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B115">
+        <v>0</v>
+      </c>
+      <c r="C115">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B116">
+        <v>0</v>
+      </c>
+      <c r="C116">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B117">
+        <v>0</v>
+      </c>
+      <c r="C117">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B118">
+        <v>0</v>
+      </c>
+      <c r="C118">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B119">
+        <v>0</v>
+      </c>
+      <c r="C119">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B120">
+        <v>0</v>
+      </c>
+      <c r="C120">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B121">
+        <v>0</v>
+      </c>
+      <c r="C121">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B122">
+        <v>0</v>
+      </c>
+      <c r="C122">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B123">
+        <v>0</v>
+      </c>
+      <c r="C123">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B124">
+        <v>0</v>
+      </c>
+      <c r="C124">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B125">
+        <v>0</v>
+      </c>
+      <c r="C125">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B126">
+        <v>0</v>
+      </c>
+      <c r="C126">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B127">
+        <v>0</v>
+      </c>
+      <c r="C127">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B129">
+        <v>2025</v>
+      </c>
+      <c r="C129">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B130">
+        <v>0</v>
+      </c>
+      <c r="C130">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B131">
+        <v>0</v>
+      </c>
+      <c r="C131">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B132">
+        <v>0</v>
+      </c>
+      <c r="C132">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B133">
+        <v>0</v>
+      </c>
+      <c r="C133">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B134">
+        <v>0</v>
+      </c>
+      <c r="C134">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B135">
+        <v>0</v>
+      </c>
+      <c r="C135">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B136">
+        <v>0</v>
+      </c>
+      <c r="C136">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B137">
+        <v>0</v>
+      </c>
+      <c r="C137">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B138">
+        <v>0</v>
+      </c>
+      <c r="C138">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B139">
+        <v>0</v>
+      </c>
+      <c r="C139">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B140">
+        <v>0</v>
+      </c>
+      <c r="C140">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B141">
+        <v>0</v>
+      </c>
+      <c r="C141">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B142">
+        <v>0</v>
+      </c>
+      <c r="C142">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B143">
+        <v>0</v>
+      </c>
+      <c r="C143">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B145">
+        <v>2025</v>
+      </c>
+      <c r="C145">
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B146">
+        <v>0</v>
+      </c>
+      <c r="C146">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B147">
+        <v>0</v>
+      </c>
+      <c r="C147">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B148">
+        <v>0</v>
+      </c>
+      <c r="C148">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B149">
+        <v>0</v>
+      </c>
+      <c r="C149">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B150">
+        <v>0</v>
+      </c>
+      <c r="C150">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B151">
+        <v>0</v>
+      </c>
+      <c r="C151">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B152">
+        <v>0</v>
+      </c>
+      <c r="C152">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B153">
+        <v>0</v>
+      </c>
+      <c r="C153">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B154">
+        <v>0</v>
+      </c>
+      <c r="C154">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B155">
+        <v>0</v>
+      </c>
+      <c r="C155">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B156">
+        <v>0</v>
+      </c>
+      <c r="C156">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B157">
+        <v>0</v>
+      </c>
+      <c r="C157">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B158">
+        <v>0</v>
+      </c>
+      <c r="C158">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>14</v>
+      </c>
+      <c r="B159">
+        <v>0</v>
+      </c>
+      <c r="C159">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
used func truncateNum to recalculatedTaxToSkuMetrics into recalculateReportsWithNewTaxRate func
</commit_message>
<xml_diff>
--- a/skuMetrics.xlsx
+++ b/skuMetrics.xlsx
@@ -465,1659 +465,1209 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C159"/>
+  <dimension ref="A1:B159"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1">
         <v>2025</v>
       </c>
-      <c r="C1">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2">
-        <v>22</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>-1072.65</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>124.62</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4">
         <v>0</v>
       </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
       <c r="B5">
-        <v>5981.06</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>11044.61</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
       <c r="B6">
         <v>0</v>
       </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
       <c r="B7">
-        <v>6656.96</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>12462.49</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
       <c r="B8">
         <v>3</v>
       </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
       <c r="B9">
-        <v>165.48</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>220.64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
       <c r="B10">
-        <v>1622.5</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>2741.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
       <c r="B11">
         <v>0</v>
       </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
       <c r="B12">
-        <v>238.91</v>
-      </c>
-      <c r="C12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
       <c r="B13">
         <v>0</v>
       </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
       <c r="B14">
-        <v>3222.82</v>
-      </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
       <c r="B15">
-        <v>48.41</v>
-      </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B17">
         <v>2025</v>
       </c>
-      <c r="C17">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>1</v>
       </c>
       <c r="B18">
-        <v>2</v>
-      </c>
-      <c r="C18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>2</v>
       </c>
       <c r="B19">
-        <v>3.4</v>
-      </c>
-      <c r="C19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>3</v>
       </c>
       <c r="B20">
         <v>0</v>
       </c>
-      <c r="C20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>4</v>
       </c>
       <c r="B21">
-        <v>375.9</v>
-      </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>5</v>
       </c>
       <c r="B22">
         <v>0</v>
       </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>6</v>
       </c>
       <c r="B23">
-        <v>340</v>
-      </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>7</v>
       </c>
       <c r="B24">
         <v>0</v>
       </c>
-      <c r="C24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>8</v>
       </c>
       <c r="B25">
-        <v>0.4</v>
-      </c>
-      <c r="C25">
-        <v>0.16</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>9</v>
       </c>
       <c r="B26">
-        <v>83.2</v>
-      </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>10</v>
       </c>
       <c r="B27">
         <v>0</v>
       </c>
-      <c r="C27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>11</v>
       </c>
       <c r="B28">
-        <v>18.03</v>
-      </c>
-      <c r="C28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>12</v>
       </c>
       <c r="B29">
         <v>0</v>
       </c>
-      <c r="C29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>13</v>
       </c>
       <c r="B30">
-        <v>158.87</v>
-      </c>
-      <c r="C30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>14</v>
       </c>
       <c r="B31">
-        <v>46.73</v>
-      </c>
-      <c r="C31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B33">
         <v>2025</v>
       </c>
-      <c r="C33">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>1</v>
       </c>
       <c r="B34">
         <v>0</v>
       </c>
-      <c r="C34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>2</v>
       </c>
       <c r="B35">
         <v>0</v>
       </c>
-      <c r="C35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>3</v>
       </c>
       <c r="B36">
         <v>0</v>
       </c>
-      <c r="C36">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>4</v>
       </c>
       <c r="B37">
         <v>0</v>
       </c>
-      <c r="C37">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>5</v>
       </c>
       <c r="B38">
         <v>0</v>
       </c>
-      <c r="C38">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>6</v>
       </c>
       <c r="B39">
         <v>0</v>
       </c>
-      <c r="C39">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>7</v>
       </c>
       <c r="B40">
         <v>0</v>
       </c>
-      <c r="C40">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>8</v>
       </c>
       <c r="B41">
         <v>0</v>
       </c>
-      <c r="C41">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>9</v>
       </c>
       <c r="B42">
         <v>0</v>
       </c>
-      <c r="C42">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>10</v>
       </c>
       <c r="B43">
         <v>0</v>
       </c>
-      <c r="C43">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>11</v>
       </c>
       <c r="B44">
         <v>0</v>
       </c>
-      <c r="C44">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>12</v>
       </c>
       <c r="B45">
         <v>0</v>
       </c>
-      <c r="C45">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>13</v>
       </c>
       <c r="B46">
         <v>0</v>
       </c>
-      <c r="C46">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>14</v>
       </c>
       <c r="B47">
         <v>0</v>
       </c>
-      <c r="C47">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B49">
         <v>2025</v>
       </c>
-      <c r="C49">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>1</v>
       </c>
       <c r="B50">
         <v>0</v>
       </c>
-      <c r="C50">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>2</v>
       </c>
       <c r="B51">
         <v>0</v>
       </c>
-      <c r="C51">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>3</v>
       </c>
       <c r="B52">
         <v>0</v>
       </c>
-      <c r="C52">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>4</v>
       </c>
       <c r="B53">
         <v>0</v>
       </c>
-      <c r="C53">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>5</v>
       </c>
       <c r="B54">
         <v>0</v>
       </c>
-      <c r="C54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>6</v>
       </c>
       <c r="B55">
         <v>0</v>
       </c>
-      <c r="C55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>7</v>
       </c>
       <c r="B56">
         <v>0</v>
       </c>
-      <c r="C56">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>8</v>
       </c>
       <c r="B57">
         <v>0</v>
       </c>
-      <c r="C57">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>9</v>
       </c>
       <c r="B58">
         <v>0</v>
       </c>
-      <c r="C58">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>10</v>
       </c>
       <c r="B59">
         <v>0</v>
       </c>
-      <c r="C59">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>11</v>
       </c>
       <c r="B60">
         <v>0</v>
       </c>
-      <c r="C60">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>12</v>
       </c>
       <c r="B61">
         <v>0</v>
       </c>
-      <c r="C61">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>13</v>
       </c>
       <c r="B62">
         <v>0</v>
       </c>
-      <c r="C62">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>14</v>
       </c>
       <c r="B63">
         <v>0</v>
       </c>
-      <c r="C63">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B65">
         <v>2025</v>
       </c>
-      <c r="C65">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>1</v>
       </c>
       <c r="B66">
-        <v>1</v>
-      </c>
-      <c r="C66">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>2</v>
       </c>
       <c r="B67">
-        <v>1.83</v>
-      </c>
-      <c r="C67">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>3</v>
       </c>
       <c r="B68">
         <v>0</v>
       </c>
-      <c r="C68">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>4</v>
       </c>
       <c r="B69">
-        <v>231.35</v>
-      </c>
-      <c r="C69">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>5</v>
       </c>
       <c r="B70">
         <v>0</v>
       </c>
-      <c r="C70">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>6</v>
       </c>
       <c r="B71">
-        <v>183</v>
-      </c>
-      <c r="C71">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>7</v>
       </c>
       <c r="B72">
         <v>0</v>
       </c>
-      <c r="C72">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>8</v>
       </c>
       <c r="B73">
         <v>0</v>
       </c>
-      <c r="C73">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>9</v>
       </c>
       <c r="B74">
-        <v>42.9</v>
-      </c>
-      <c r="C74">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>10</v>
       </c>
       <c r="B75">
         <v>0</v>
       </c>
-      <c r="C75">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>11</v>
       </c>
       <c r="B76">
-        <v>13.24</v>
-      </c>
-      <c r="C76">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>12</v>
       </c>
       <c r="B77">
         <v>0</v>
       </c>
-      <c r="C77">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>13</v>
       </c>
       <c r="B78">
-        <v>117.38</v>
-      </c>
-      <c r="C78">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>14</v>
       </c>
       <c r="B79">
-        <v>64.14</v>
-      </c>
-      <c r="C79">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B81">
         <v>2025</v>
       </c>
-      <c r="C81">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>1</v>
       </c>
       <c r="B82">
-        <v>1</v>
-      </c>
-      <c r="C82">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>2</v>
       </c>
       <c r="B83">
-        <v>1.83</v>
-      </c>
-      <c r="C83">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>3</v>
       </c>
       <c r="B84">
         <v>0</v>
       </c>
-      <c r="C84">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>4</v>
       </c>
       <c r="B85">
-        <v>231.35</v>
-      </c>
-      <c r="C85">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>5</v>
       </c>
       <c r="B86">
         <v>0</v>
       </c>
-      <c r="C86">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>6</v>
       </c>
       <c r="B87">
-        <v>183</v>
-      </c>
-      <c r="C87">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>7</v>
       </c>
       <c r="B88">
         <v>0</v>
       </c>
-      <c r="C88">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>8</v>
       </c>
       <c r="B89">
         <v>0</v>
       </c>
-      <c r="C89">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>9</v>
       </c>
       <c r="B90">
-        <v>42.9</v>
-      </c>
-      <c r="C90">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>10</v>
       </c>
       <c r="B91">
         <v>0</v>
       </c>
-      <c r="C91">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>11</v>
       </c>
       <c r="B92">
-        <v>13.24</v>
-      </c>
-      <c r="C92">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>12</v>
       </c>
       <c r="B93">
         <v>0</v>
       </c>
-      <c r="C93">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>13</v>
       </c>
       <c r="B94">
-        <v>117.38</v>
-      </c>
-      <c r="C94">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>14</v>
       </c>
       <c r="B95">
-        <v>64.14</v>
-      </c>
-      <c r="C95">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B97">
         <v>2025</v>
       </c>
-      <c r="C97">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>1</v>
       </c>
       <c r="B98">
-        <v>14</v>
-      </c>
-      <c r="C98">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>2</v>
       </c>
       <c r="B99">
-        <v>-606.4</v>
-      </c>
-      <c r="C99">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+        <v>57.76</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>3</v>
       </c>
       <c r="B100">
         <v>0</v>
       </c>
-      <c r="C100">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>4</v>
       </c>
       <c r="B101">
-        <v>3215.06</v>
-      </c>
-      <c r="C101">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+        <v>4579.93</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>5</v>
       </c>
       <c r="B102">
         <v>0</v>
       </c>
-      <c r="C102">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>6</v>
       </c>
       <c r="B103">
-        <v>4048</v>
-      </c>
-      <c r="C103">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5776.51</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>7</v>
       </c>
       <c r="B104">
         <v>3</v>
       </c>
-      <c r="C104">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>8</v>
       </c>
       <c r="B105">
-        <v>176.96</v>
-      </c>
-      <c r="C105">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+        <v>252.42</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>9</v>
       </c>
       <c r="B106">
-        <v>1151.3</v>
-      </c>
-      <c r="C106">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+        <v>1504.7</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>10</v>
       </c>
       <c r="B107">
         <v>0</v>
       </c>
-      <c r="C107">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>11</v>
       </c>
       <c r="B108">
-        <v>110.28</v>
-      </c>
-      <c r="C108">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>12</v>
       </c>
       <c r="B109">
         <v>0</v>
       </c>
-      <c r="C109">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>13</v>
       </c>
       <c r="B110">
-        <v>1598.92</v>
-      </c>
-      <c r="C110">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>14</v>
       </c>
       <c r="B111">
-        <v>39.5</v>
-      </c>
-      <c r="C111">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B113">
         <v>2025</v>
       </c>
-      <c r="C113">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>1</v>
       </c>
       <c r="B114">
         <v>0</v>
       </c>
-      <c r="C114">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>2</v>
       </c>
       <c r="B115">
         <v>0</v>
       </c>
-      <c r="C115">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>3</v>
       </c>
       <c r="B116">
         <v>0</v>
       </c>
-      <c r="C116">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>4</v>
       </c>
       <c r="B117">
         <v>0</v>
       </c>
-      <c r="C117">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>5</v>
       </c>
       <c r="B118">
         <v>0</v>
       </c>
-      <c r="C118">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>6</v>
       </c>
       <c r="B119">
         <v>0</v>
       </c>
-      <c r="C119">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>7</v>
       </c>
       <c r="B120">
         <v>0</v>
       </c>
-      <c r="C120">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>8</v>
       </c>
       <c r="B121">
         <v>0</v>
       </c>
-      <c r="C121">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>9</v>
       </c>
       <c r="B122">
         <v>0</v>
       </c>
-      <c r="C122">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>10</v>
       </c>
       <c r="B123">
         <v>0</v>
       </c>
-      <c r="C123">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>11</v>
       </c>
       <c r="B124">
         <v>0</v>
       </c>
-      <c r="C124">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>12</v>
       </c>
       <c r="B125">
         <v>0</v>
       </c>
-      <c r="C125">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>13</v>
       </c>
       <c r="B126">
         <v>0</v>
       </c>
-      <c r="C126">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>14</v>
       </c>
       <c r="B127">
         <v>0</v>
       </c>
-      <c r="C127">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B129">
         <v>2025</v>
       </c>
-      <c r="C129">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>1</v>
       </c>
       <c r="B130">
         <v>0</v>
       </c>
-      <c r="C130">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>2</v>
       </c>
       <c r="B131">
         <v>0</v>
       </c>
-      <c r="C131">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>3</v>
       </c>
       <c r="B132">
         <v>0</v>
       </c>
-      <c r="C132">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>4</v>
       </c>
       <c r="B133">
         <v>0</v>
       </c>
-      <c r="C133">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>5</v>
       </c>
       <c r="B134">
         <v>0</v>
       </c>
-      <c r="C134">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>6</v>
       </c>
       <c r="B135">
         <v>0</v>
       </c>
-      <c r="C135">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>7</v>
       </c>
       <c r="B136">
         <v>0</v>
       </c>
-      <c r="C136">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>8</v>
       </c>
       <c r="B137">
         <v>0</v>
       </c>
-      <c r="C137">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>9</v>
       </c>
       <c r="B138">
         <v>0</v>
       </c>
-      <c r="C138">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>10</v>
       </c>
       <c r="B139">
         <v>0</v>
       </c>
-      <c r="C139">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>11</v>
       </c>
       <c r="B140">
         <v>0</v>
       </c>
-      <c r="C140">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>12</v>
       </c>
       <c r="B141">
         <v>0</v>
       </c>
-      <c r="C141">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>13</v>
       </c>
       <c r="B142">
         <v>0</v>
       </c>
-      <c r="C142">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>14</v>
       </c>
       <c r="B143">
         <v>0</v>
       </c>
-      <c r="C143">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B145">
         <v>2025</v>
       </c>
-      <c r="C145">
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>1</v>
       </c>
       <c r="B146">
         <v>0</v>
       </c>
-      <c r="C146">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>2</v>
       </c>
       <c r="B147">
         <v>0</v>
       </c>
-      <c r="C147">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>3</v>
       </c>
       <c r="B148">
         <v>0</v>
       </c>
-      <c r="C148">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>4</v>
       </c>
       <c r="B149">
         <v>0</v>
       </c>
-      <c r="C149">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>5</v>
       </c>
       <c r="B150">
         <v>0</v>
       </c>
-      <c r="C150">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>6</v>
       </c>
       <c r="B151">
         <v>0</v>
       </c>
-      <c r="C151">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>7</v>
       </c>
       <c r="B152">
         <v>0</v>
       </c>
-      <c r="C152">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>8</v>
       </c>
       <c r="B153">
         <v>0</v>
       </c>
-      <c r="C153">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>9</v>
       </c>
       <c r="B154">
         <v>0</v>
       </c>
-      <c r="C154">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>10</v>
       </c>
       <c r="B155">
         <v>0</v>
       </c>
-      <c r="C155">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>11</v>
       </c>
       <c r="B156">
         <v>0</v>
       </c>
-      <c r="C156">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>12</v>
       </c>
       <c r="B157">
         <v>0</v>
       </c>
-      <c r="C157">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>13</v>
       </c>
       <c r="B158">
         <v>0</v>
       </c>
-      <c r="C158">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>14</v>
       </c>
       <c r="B159">
-        <v>0</v>
-      </c>
-      <c r="C159">
         <v>0</v>
       </c>
     </row>

</xml_diff>